<commit_message>
docs: add survey sheets to example workbooks
</commit_message>
<xml_diff>
--- a/test_data/examples/wildcat/wildcat_workbook.xlsx
+++ b/test_data/examples/wildcat/wildcat_workbook.xlsx
@@ -10,11 +10,12 @@
     <sheet name="Metadata" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Header" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="GridPolicy" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="HoleCasings" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Plugs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Stratigraphy" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SubsurfaceAssumptions" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Survey" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="HoleCasings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Plugs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Stratigraphy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SubsurfaceAssumptions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Notes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -722,325 +723,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>md_rkb</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>inclination_deg</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>top_rkb</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>bottom_rkb</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>diameter_in</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>shoe</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>hc_perm</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Hole 36 in</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>hole</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>132</v>
-      </c>
-      <c r="D2" t="n">
-        <v>190</v>
-      </c>
-      <c r="E2" t="n">
-        <v>36</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hole 26 in</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>hole</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>190</v>
-      </c>
-      <c r="D3" t="n">
-        <v>444</v>
-      </c>
-      <c r="E3" t="n">
-        <v>26</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Hole 17 1/2 in</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>hole</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>444</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1812</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>17 1/2</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Hole 12 1/4 in</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>hole</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>1812</v>
-      </c>
-      <c r="D5" t="n">
-        <v>3942</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>12 1/4</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Hole 8 1/2 in</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>hole</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>3942</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3997</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>8 1/2</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Casing 30 in</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>casing</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>132</v>
-      </c>
-      <c r="D7" t="n">
-        <v>158</v>
-      </c>
-      <c r="E7" t="n">
-        <v>30</v>
-      </c>
-      <c r="F7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Cement 30 in</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>casing cement</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>132</v>
-      </c>
-      <c r="D8" t="n">
-        <v>158</v>
-      </c>
-      <c r="E8" t="n">
-        <v>30</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Casing 20 in</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>casing</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>132</v>
-      </c>
-      <c r="D9" t="n">
-        <v>439</v>
-      </c>
-      <c r="E9" t="n">
-        <v>20</v>
-      </c>
-      <c r="F9" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Cement 20 in</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>casing cement</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>132</v>
-      </c>
-      <c r="D10" t="n">
-        <v>439</v>
-      </c>
-      <c r="E10" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Casing 13 3/8 in</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>casing</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>182</v>
-      </c>
-      <c r="D11" t="n">
-        <v>1803</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>13 3/8</t>
-        </is>
-      </c>
-      <c r="F11" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Cement 13 3/8 in</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>casing cement</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>450</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1803</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>13 3/8</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
-        <v>500</v>
+          <t>azimuth_deg</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1054,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1080,71 +780,299 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>cement_perm</t>
+          <t>diameter_in</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>shoe</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>hc_perm</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>cplug3</t>
+          <t>Hole 36 in</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>cement</t>
+          <t>hole</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>132</v>
       </c>
       <c r="D2" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cplug2</t>
+          <t>Hole 26 in</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cement</t>
+          <t>hole</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1690</v>
+        <v>190</v>
       </c>
       <c r="D3" t="n">
-        <v>1850</v>
+        <v>444</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cplug1</t>
+          <t>Hole 17 1/2 in</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>cement</t>
+          <t>hole</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2050</v>
+        <v>444</v>
       </c>
       <c r="D4" t="n">
-        <v>2300</v>
-      </c>
-      <c r="E4" t="n">
-        <v>5</v>
+        <v>1812</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>17 1/2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hole 12 1/4 in</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>hole</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1812</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3942</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>12 1/4</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hole 8 1/2 in</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hole</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3942</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3997</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>8 1/2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Casing 30 in</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>casing</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>132</v>
+      </c>
+      <c r="D7" t="n">
+        <v>158</v>
+      </c>
+      <c r="E7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cement 30 in</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>casing cement</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>132</v>
+      </c>
+      <c r="D8" t="n">
+        <v>158</v>
+      </c>
+      <c r="E8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Casing 20 in</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>casing</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>132</v>
+      </c>
+      <c r="D9" t="n">
+        <v>439</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cement 20 in</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>casing cement</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>132</v>
+      </c>
+      <c r="D10" t="n">
+        <v>439</v>
+      </c>
+      <c r="E10" t="n">
+        <v>20</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Casing 13 3/8 in</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>casing</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>182</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1803</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>13 3/8</t>
+        </is>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cement 13 3/8 in</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>casing cement</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>450</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1803</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>13 3/8</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -1158,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1169,234 +1097,86 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>top_rkb</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>bottom_rkb</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>unit_type</t>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cement_perm</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NORDLAND GP</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+          <t>cplug3</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>cement</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>132</v>
       </c>
-      <c r="C2" t="n">
-        <v>544</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
+      <c r="D2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HORDALAND GP</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>544</v>
+          <t>cplug2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>cement</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>1041</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
+        <v>1690</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1850</v>
+      </c>
+      <c r="E3" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ROGALAND GP</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1041</v>
+          <t>cplug1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>cement</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>1163</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SHETLAND GP</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1163</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1444</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CROMER KNOLL GP</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1444</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2122</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>VIKING GP</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2122</v>
-      </c>
-      <c r="C7" t="n">
-        <v>2265</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>JURASSIC SS</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2265</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2352</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>reservoir</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>SKAGERRAK FM</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>2352</v>
-      </c>
-      <c r="C9" t="n">
-        <v>2532</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>reservoir</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SMITH BANK FM</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>2532</v>
-      </c>
-      <c r="C10" t="n">
-        <v>2665</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>reservoir</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ZECHSTEIN GP</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2665</v>
-      </c>
-      <c r="C11" t="n">
-        <v>3829</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>KUPFERSCHIEFER FM</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>3829</v>
-      </c>
-      <c r="C12" t="n">
-        <v>3834</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ROTLIEGEND GP</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>3834</v>
-      </c>
-      <c r="C13" t="n">
-        <v>3997</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>undefined</t>
-        </is>
+        <v>2050</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2300</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1410,69 +1190,245 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>temperature_gradient</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>ground_temperature</t>
+          <t>top_rkb</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>fluid_type</t>
+          <t>bottom_rkb</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>z_fluid_contact</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>p_fluid_contact</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>z_resrv</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>p_resrv</t>
+          <t>unit_type</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>31</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NORDLAND GP</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>co2</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>2400</v>
-      </c>
-      <c r="E2" t="n">
-        <v>245</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2450</v>
-      </c>
-      <c r="G2" t="n">
-        <v>250</v>
+        <v>132</v>
+      </c>
+      <c r="C2" t="n">
+        <v>544</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HORDALAND GP</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>544</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1041</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ROGALAND GP</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1041</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1163</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SHETLAND GP</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1163</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1444</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CROMER KNOLL GP</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1444</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2122</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VIKING GP</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2122</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2265</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>JURASSIC SS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2265</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2352</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>reservoir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SKAGERRAK FM</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2352</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2532</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>reservoir</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SMITH BANK FM</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2532</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2665</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>reservoir</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ZECHSTEIN GP</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2665</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3829</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>KUPFERSCHIEFER FM</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3829</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3834</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ROTLIEGEND GP</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3834</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3997</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>undefined</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1486,12 +1442,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>temperature_gradient</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ground_temperature</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fluid_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>z_fluid_contact</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>p_fluid_contact</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>z_resrv</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>p_resrv</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>co2</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E2" t="n">
+        <v>245</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G2" t="n">
+        <v>250</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -1506,12 +1538,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GridPolicy and SubsurfaceAssumptions are editable example scenario values and must be reviewed for a real case.</t>
+          <t>Survey is optional: leave it empty for vertical wells or add md_rkb, inclination_deg, and azimuth_deg rows for deviation.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
+        <is>
+          <t>GridPolicy and SubsurfaceAssumptions are editable example scenario values and must be reviewed for a real case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>z_fluid_contact and p_fluid_contact define the GAS_WATER datum and WGC depth in CIRRUS.</t>
         </is>

</xml_diff>